<commit_message>
feat(s0-b02): add shared design tokens and visual QA
</commit_message>
<xml_diff>
--- a/AI_Marketing_Platform_Engineering_Master_Backlog_2_Developers_v1.1.xlsx
+++ b/AI_Marketing_Platform_Engineering_Master_Backlog_2_Developers_v1.1.xlsx
@@ -19569,7 +19569,7 @@
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="15" ht="155.1" customHeight="1" s="48">
+    <s:row r="15" ht="210" customHeight="1" s="48">
       <s:c r="A15" s="17" t="inlineStr">
         <s:is>
           <s:t>S0-B02</s:t>
@@ -19625,7 +19625,7 @@
       </s:c>
       <s:c r="L15" s="28" t="inlineStr">
         <s:is>
-          <s:t>In Progress</s:t>
+          <s:t>In Review</s:t>
         </s:is>
       </s:c>
       <s:c r="M15" s="13" t="inlineStr">
@@ -19658,7 +19658,7 @@
       </s:c>
       <s:c r="S15" s="29" t="inlineStr">
         <s:is>
-          <s:t>docs/backlog-deep-audit-2026-09-07.json#S0-B02</s:t>
+          <s:t>docs/S0-B02-REPORT-SQ.md</s:t>
         </s:is>
       </s:c>
       <s:c r="T15" s="13" t="inlineStr">
@@ -19688,42 +19688,43 @@
       </s:c>
       <s:c r="Y15" s="54" t="inlineStr">
         <s:is>
-          <s:t>Pjesërisht</s:t>
+          <s:t>Në review</s:t>
         </s:is>
       </s:c>
       <s:c r="Z15" s="55" t="inlineStr">
         <s:is>
-          <s:t>Temë Nuxt UI, light/dark, Inter lokal, ikona lokale dhe logo SVG transparente; dashboard dhe landing të unifikuara.</s:t>
+          <s:t>U vendos kontrata e përbashkët `--rrit-*` për ngjyra semantike, tipografi, hapësirë, radius, hije dhe motion. Landing dhe dashboard konsumojnë tokenat e UI-së; Nuxt UI v4, Lucide dhe politika e wrapper-ave janë të dokumentuara. Light/dark tokenat dhe testet accessibility u shtuan.</s:t>
         </s:is>
       </s:c>
       <s:c r="AA15" s="55" t="inlineStr">
         <s:is>
-          <s:t>1. Ka ende konstante stili në komponentë; duhet rishikim kontrasti/dark mode dhe provë vizuale e versionit aktual.</s:t>
+          <s:t>Mbeten GitHub Actions në PR, review i Programmer A dhe RG-14. Testi i dashboard accessibility krijon të dhëna sintetike dhe duhet të ekzekutohet vetëm në ambient të dedikuar/CI, jo kundër Supabase v1.</s:t>
         </s:is>
       </s:c>
       <s:c r="AB15" s="55" t="inlineStr">
         <s:is>
-          <s:t>Prova e kërkuar nga backlog-u: Vitest/component visual QA
-Kriteri për t'u verifikuar (nuk deklarohet i kaluar): Tokens drive landing and dashboard; no random feature-level design constants; contrast baseline passes; dark mode has no unreadable states.
-Pranimi kërkon edhe gate-et: RG-14. Asnjë gate nuk është shënuar Passed nga ky audit.</s:t>
+          <s:t>Kriteri lokal i verifikuar: tokenat përdoren për UI standarde në landing dhe dashboard; light/dark accessibility baseline kalon për landing. Ilustrimet e landing-ut lejohen të mbajnë ngjyra/gradientë lokalë sepse janë art-direction, jo konstante të UI-së. RG-14 nuk është shënuar Passed.</s:t>
         </s:is>
       </s:c>
       <s:c r="AC15" s="55" t="inlineStr">
         <s:is>
-          <s:t>hq-deep-audit-lint.log, hq-deep-audit-app-types.log, hq-deep-audit-server-types.log: exit 0; lint i plotë dhe TypeScript app/server. Nuk u krye clean install/build prodhimi ose hosted CI.</s:t>
+          <s:t>2026-09-09: `npm.cmd run check` kaloi (toolchain, ESLint, Nuxt typecheck, 27/27 Vitest unit); `npm.cmd run build` kaloi; Playwright landing desktop kaloi 13/13 me kontroll light/dark. `git diff --check` kaloi.</s:t>
         </s:is>
       </s:c>
       <s:c r="AD15" s="55" t="inlineStr">
         <s:is>
-          <s:t>apps/web/app/app.config.ts
-apps/web/app/assets/css/main.css
-apps/web/app/components/BrandLogo.vue
-docs/UI-SYSTEM.md</s:t>
+          <s:t>apps/web/app/assets/css/main.css
+apps/web/app/assets/css/landing.css
+apps/web/app/utils/design-system.ts
+apps/web/app/app.config.ts
+apps/web/tests/unit/design-system.test.ts
+apps/web/tests/e2e/accessibility-baseline.spec.ts
+docs/S0-B02-REPORT-SQ.md</s:t>
         </s:is>
       </s:c>
       <s:c r="AE15" s="42" t="inlineStr">
         <s:is>
-          <s:t>Pjesërisht — kërkon zhvillim</s:t>
+          <s:t>Në review — implementimi dhe validimi lokal u kryen; CI/review/RG-14 mbeten.</s:t>
         </s:is>
       </s:c>
       <s:c r="AF15" s="42" t="inlineStr">

</xml_diff>